<commit_message>
cancer incid + dis duration
</commit_message>
<xml_diff>
--- a/output/Tables/7000 steps/HIA_7000steps_1000replicate.xlsx
+++ b/output/Tables/7000 steps/HIA_7000steps_1000replicate.xlsx
@@ -1,108 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ines/Documents/PhD/PROJETS/MARCHE/HIA_walking_steps/output/Tables/7000 steps/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569CCBBD-D9C9-1C49-BDF7-ABA599CB688D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
-  <si>
-    <t>disease</t>
-  </si>
-  <si>
-    <t>tot_cases</t>
-  </si>
-  <si>
-    <t>tot_cases_low</t>
-  </si>
-  <si>
-    <t>tot_cases_up</t>
-  </si>
-  <si>
-    <t>tot_daly</t>
-  </si>
-  <si>
-    <t>tot_daly_low</t>
-  </si>
-  <si>
-    <t>tot_daly_up</t>
-  </si>
-  <si>
-    <t>tot_medic_costs</t>
-  </si>
-  <si>
-    <t>tot_medic_costs_low</t>
-  </si>
-  <si>
-    <t>tot_medic_costs_up</t>
-  </si>
-  <si>
-    <t>tot_soc_costs</t>
-  </si>
-  <si>
-    <t>tot_soc_costs_low</t>
-  </si>
-  <si>
-    <t>tot_soc_costs_up</t>
-  </si>
-  <si>
-    <t>mort</t>
-  </si>
-  <si>
-    <t>cvd</t>
-  </si>
-  <si>
-    <t>cancer</t>
-  </si>
-  <si>
-    <t>diab2</t>
-  </si>
-  <si>
-    <t>dem</t>
-  </si>
-  <si>
-    <t>dep</t>
-  </si>
-  <si>
-    <t>Morbidity</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -202,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -236,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -271,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -447,72 +350,100 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>13</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases_low</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases_up</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly_low</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly_up</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs_low</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs_up</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs_low</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs_up</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mort</t>
+        </is>
       </c>
       <c r="B2">
-        <v>158929.88399999999</v>
+        <v>167177.387</v>
       </c>
       <c r="C2">
-        <v>153673.755</v>
+        <v>161731.654</v>
       </c>
       <c r="D2">
-        <v>164168.66500000001</v>
+        <v>172619.933</v>
       </c>
       <c r="E2">
-        <v>1652111.443</v>
+        <v>1638288.598</v>
       </c>
       <c r="F2">
-        <v>1626354.818</v>
+        <v>1613068.99</v>
       </c>
       <c r="G2">
-        <v>1678001.52</v>
+        <v>1663591.834</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -524,200 +455,210 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>219734230443.47101</v>
+        <v>217896358939.252</v>
       </c>
       <c r="L2">
-        <v>216282696938.04099</v>
+        <v>214523681362.054</v>
       </c>
       <c r="M2">
-        <v>223166621312.996</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>14</v>
+        <v>221259380208.131</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cvd</t>
+        </is>
       </c>
       <c r="B3">
-        <v>145867.71799999999</v>
+        <v>133604.203</v>
       </c>
       <c r="C3">
-        <v>142431.788</v>
+        <v>130501.029</v>
       </c>
       <c r="D3">
-        <v>149296.17800000001</v>
+        <v>136693.187</v>
       </c>
       <c r="E3">
-        <v>130654</v>
+        <v>181819.296</v>
       </c>
       <c r="F3">
-        <v>128078.64200000001</v>
+        <v>178196.008</v>
       </c>
       <c r="G3">
-        <v>133250.74299999999</v>
+        <v>185472.025</v>
       </c>
       <c r="H3">
-        <v>8124698949.3789997</v>
+        <v>7040133264.596</v>
       </c>
       <c r="I3">
-        <v>7934956490.224</v>
+        <v>6877832945.504</v>
       </c>
       <c r="J3">
-        <v>8316918714.9709997</v>
+        <v>7203906875.536</v>
       </c>
       <c r="K3">
-        <v>17377593706.162998</v>
+        <v>24182097205.912</v>
       </c>
       <c r="L3">
-        <v>17033452205.992001</v>
+        <v>23697745075.115</v>
       </c>
       <c r="M3">
-        <v>17719265773.078999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>15</v>
+        <v>24669155799.566</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cancer</t>
+        </is>
       </c>
       <c r="B4">
-        <v>130156.452</v>
+        <v>29791.03</v>
       </c>
       <c r="C4">
-        <v>127339.19500000001</v>
+        <v>29107.405</v>
       </c>
       <c r="D4">
-        <v>133001.75700000001</v>
+        <v>30480.033</v>
       </c>
       <c r="E4">
-        <v>194056.86900000001</v>
+        <v>13856.512</v>
       </c>
       <c r="F4">
-        <v>188514.32500000001</v>
+        <v>13567.106</v>
       </c>
       <c r="G4">
-        <v>199727.66500000001</v>
+        <v>14150.966</v>
       </c>
       <c r="H4">
-        <v>1927333900.4389999</v>
+        <v>873455050.115</v>
       </c>
       <c r="I4">
-        <v>1885504675.3410001</v>
+        <v>853390435.5700001</v>
       </c>
       <c r="J4">
-        <v>1969531353.132</v>
+        <v>893849476.7640001</v>
       </c>
       <c r="K4">
-        <v>25809224695.313999</v>
+        <v>1842939290.754</v>
       </c>
       <c r="L4">
-        <v>25073546427.196999</v>
+        <v>1804464463.578</v>
       </c>
       <c r="M4">
-        <v>26563554289.839001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>16</v>
+        <v>1882037482.607</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>diab2</t>
+        </is>
       </c>
       <c r="B5">
-        <v>27773.387999999999</v>
+        <v>20459.467</v>
       </c>
       <c r="C5">
-        <v>27143.224999999999</v>
+        <v>20074.98</v>
       </c>
       <c r="D5">
-        <v>28411.325000000001</v>
+        <v>20847.956</v>
       </c>
       <c r="E5">
-        <v>54678.493999999999</v>
+        <v>37567.92</v>
       </c>
       <c r="F5">
-        <v>53339.87</v>
+        <v>36830.167</v>
       </c>
       <c r="G5">
-        <v>56050.934999999998</v>
+        <v>38323.856</v>
       </c>
       <c r="H5">
-        <v>2088559330.277</v>
+        <v>802018195.166</v>
       </c>
       <c r="I5">
-        <v>2041340486.7160001</v>
+        <v>786959315.9630001</v>
       </c>
       <c r="J5">
-        <v>2136670347.0899999</v>
+        <v>817301832.9400001</v>
       </c>
       <c r="K5">
-        <v>7271900219.4700003</v>
+        <v>4996532261.015</v>
       </c>
       <c r="L5">
-        <v>7093342931.1520004</v>
+        <v>4898685908.956</v>
       </c>
       <c r="M5">
-        <v>7454918231.8149996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>17</v>
+        <v>5096633827.326</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dem</t>
+        </is>
       </c>
       <c r="B6">
-        <v>51067.036</v>
+        <v>48264.267</v>
       </c>
       <c r="C6">
-        <v>49167.858999999997</v>
+        <v>46518.77</v>
       </c>
       <c r="D6">
-        <v>52976.908000000003</v>
+        <v>50022.045</v>
       </c>
       <c r="E6">
-        <v>81803.156000000003</v>
+        <v>55223.729</v>
       </c>
       <c r="F6">
-        <v>79573.919999999998</v>
+        <v>53186.786</v>
       </c>
       <c r="G6">
-        <v>84042.527000000002</v>
+        <v>57282.696</v>
       </c>
       <c r="H6">
-        <v>859803645.36199999</v>
+        <v>803399869.79</v>
       </c>
       <c r="I6">
-        <v>828081835.05799997</v>
+        <v>774550346.541</v>
       </c>
       <c r="J6">
-        <v>891700649.25100005</v>
+        <v>832395632.997</v>
       </c>
       <c r="K6">
-        <v>10879431502.521999</v>
+        <v>7344722306.631</v>
       </c>
       <c r="L6">
-        <v>10581296787.228001</v>
+        <v>7072294081.077</v>
       </c>
       <c r="M6">
-        <v>11178553935.142</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>18</v>
+        <v>7617927048.053</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dep</t>
+        </is>
       </c>
       <c r="B7">
-        <v>511592.73700000002</v>
+        <v>439884.178</v>
       </c>
       <c r="C7">
-        <v>503679.397</v>
+        <v>433830.81</v>
       </c>
       <c r="D7">
-        <v>519587.80499999999</v>
+        <v>445921.129</v>
       </c>
       <c r="E7">
-        <v>164673.163</v>
+        <v>160643.367</v>
       </c>
       <c r="F7">
-        <v>160516.57</v>
+        <v>157049.226</v>
       </c>
       <c r="G7">
-        <v>168897.557</v>
+        <v>164259.11</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -729,95 +670,99 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>21901945200.855999</v>
+        <v>21366641969.324</v>
       </c>
       <c r="L7">
-        <v>21348713699.119999</v>
+        <v>20887176186.423</v>
       </c>
       <c r="M7">
-        <v>22464961459.577999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>19</v>
+        <v>21847774873.213</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Morbidity</t>
+        </is>
       </c>
       <c r="B8">
-        <v>866457.33100000001</v>
+        <v>672003.145</v>
       </c>
       <c r="C8">
-        <v>849761.46399999992</v>
+        <v>660032.9939999999</v>
       </c>
       <c r="D8">
-        <v>883273.973</v>
+        <v>683964.3500000001</v>
       </c>
       <c r="E8">
-        <v>625865.68200000003</v>
+        <v>449110.824</v>
       </c>
       <c r="F8">
-        <v>610023.32700000005</v>
+        <v>438829.2930000001</v>
       </c>
       <c r="G8">
-        <v>641969.42700000003</v>
+        <v>459488.653</v>
       </c>
       <c r="H8">
-        <v>13000395825.457001</v>
+        <v>9519006379.667</v>
       </c>
       <c r="I8">
-        <v>12689883487.339001</v>
+        <v>9292733043.577999</v>
       </c>
       <c r="J8">
-        <v>13314821064.444</v>
+        <v>9747453818.237</v>
       </c>
       <c r="K8">
-        <v>83240095324.324997</v>
+        <v>59732933033.636</v>
       </c>
       <c r="L8">
-        <v>81130352050.688995</v>
+        <v>58360365715.149</v>
       </c>
       <c r="M8">
-        <v>85381253689.453003</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>20</v>
+        <v>61113529030.765</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
       </c>
       <c r="B9">
-        <v>1025387.215</v>
+        <v>839180.532</v>
       </c>
       <c r="C9">
-        <v>1003435.219</v>
+        <v>821764.648</v>
       </c>
       <c r="D9">
-        <v>1047442.638</v>
+        <v>856584.2830000001</v>
       </c>
       <c r="E9">
-        <v>2277977.125</v>
+        <v>2087399.422</v>
       </c>
       <c r="F9">
-        <v>2236378.145</v>
+        <v>2051898.283</v>
       </c>
       <c r="G9">
-        <v>2319970.9470000002</v>
+        <v>2123080.487</v>
       </c>
       <c r="H9">
-        <v>13000395825.457001</v>
+        <v>9519006379.667</v>
       </c>
       <c r="I9">
-        <v>12689883487.339001</v>
+        <v>9292733043.577999</v>
       </c>
       <c r="J9">
-        <v>13314821064.444</v>
+        <v>9747453818.237</v>
       </c>
       <c r="K9">
-        <v>302974325767.79602</v>
+        <v>277629291972.888</v>
       </c>
       <c r="L9">
-        <v>297413048988.72998</v>
+        <v>272884047077.203</v>
       </c>
       <c r="M9">
-        <v>308547875002.44897</v>
+        <v>282372909238.896</v>
       </c>
     </row>
   </sheetData>

</xml_diff>